<commit_message>
primer excel generado, esta en mitad de proceso a que salga bien
</commit_message>
<xml_diff>
--- a/backend/templates/excel/plantilla_1.xlsx
+++ b/backend/templates/excel/plantilla_1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Descargas\SAN PEDRO 11 MAR JUAN CAMILO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecnologicodeantioquia-my.sharepoint.com/personal/paola_garcia44_correo_tdea_edu_co/Documents/Escritorio/Automatización geotecnica/automatizacion_geotecnica/backend/templates/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622C883C-C2C7-4B70-A3F0-C530FA572C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{622C883C-C2C7-4B70-A3F0-C530FA572C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{580A2FF4-72AA-40C2-ADF3-121DE9D6F21A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -878,6 +878,37 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -914,6 +945,15 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -959,46 +999,6 @@
     <xf numFmtId="2" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1034,14 +1034,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>630114</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>8918</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>258639</xdr:colOff>
+      <xdr:colOff>399443</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>134974</xdr:rowOff>
     </xdr:to>
@@ -1072,8 +1072,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9344268" y="0"/>
-          <a:ext cx="5724525" cy="5870575"/>
+          <a:off x="9094940" y="0"/>
+          <a:ext cx="5724525" cy="5957648"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1433,177 +1433,177 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="47"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="60"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="Q2" s="61"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="48"/>
-      <c r="P3" s="48"/>
-      <c r="Q3" s="48"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="62"/>
+      <c r="Q3" s="62"/>
     </row>
     <row r="4" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="49"/>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
-      <c r="K4" s="50"/>
-      <c r="L4" s="50"/>
-      <c r="M4" s="50"/>
-      <c r="N4" s="50"/>
-      <c r="O4" s="50"/>
-      <c r="P4" s="50"/>
-      <c r="Q4" s="51"/>
+      <c r="A4" s="63"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="64"/>
+      <c r="M4" s="64"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="65"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="53" t="s">
+      <c r="B5" s="66"/>
+      <c r="C5" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="53"/>
-      <c r="N5" s="53"/>
-      <c r="O5" s="53"/>
-      <c r="P5" s="53"/>
-      <c r="Q5" s="53"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="67"/>
+      <c r="F5" s="67"/>
+      <c r="G5" s="67"/>
+      <c r="H5" s="67"/>
+      <c r="I5" s="67"/>
+      <c r="J5" s="67"/>
+      <c r="K5" s="67"/>
+      <c r="L5" s="67"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="67"/>
     </row>
     <row r="6" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="54" t="s">
+      <c r="B6" s="66"/>
+      <c r="C6" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="54"/>
-      <c r="N6" s="54"/>
-      <c r="O6" s="54"/>
-      <c r="P6" s="54"/>
-      <c r="Q6" s="54"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="68"/>
+      <c r="N6" s="68"/>
+      <c r="O6" s="68"/>
+      <c r="P6" s="68"/>
+      <c r="Q6" s="68"/>
     </row>
     <row r="7" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="34">
+      <c r="B7" s="72"/>
+      <c r="C7" s="45">
         <v>46112</v>
       </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="36" t="s">
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="36"/>
+      <c r="G7" s="47"/>
       <c r="H7" s="10">
         <v>63.5</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="37" t="s">
+      <c r="J7" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="37"/>
-      <c r="L7" s="38" t="s">
+      <c r="K7" s="48"/>
+      <c r="L7" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="39"/>
-      <c r="N7" s="55" t="s">
+      <c r="M7" s="50"/>
+      <c r="N7" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="56"/>
-      <c r="P7" s="56"/>
-      <c r="Q7" s="57"/>
+      <c r="O7" s="70"/>
+      <c r="P7" s="70"/>
+      <c r="Q7" s="71"/>
     </row>
     <row r="8" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="42" t="s">
+      <c r="B8" s="72"/>
+      <c r="C8" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="43"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="36" t="s">
+      <c r="D8" s="54"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="36"/>
+      <c r="G8" s="47"/>
       <c r="H8" s="10">
         <v>0.76</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="37"/>
-      <c r="K8" s="37"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="41"/>
-      <c r="N8" s="55" t="s">
+      <c r="J8" s="48"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="52"/>
+      <c r="N8" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="O8" s="56"/>
-      <c r="P8" s="56"/>
-      <c r="Q8" s="57"/>
+      <c r="O8" s="70"/>
+      <c r="P8" s="70"/>
+      <c r="Q8" s="71"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -1662,7 +1662,7 @@
       <c r="A10" s="14">
         <v>0.45</v>
       </c>
-      <c r="B10" s="65">
+      <c r="B10" s="38">
         <v>15</v>
       </c>
       <c r="C10" s="14">
@@ -1677,7 +1677,7 @@
         <f t="shared" ref="E10:E16" si="1">C10-D10</f>
         <v>6.75</v>
       </c>
-      <c r="F10" s="60">
+      <c r="F10" s="33">
         <v>7</v>
       </c>
       <c r="G10" s="16">
@@ -1719,7 +1719,7 @@
         <f>L10</f>
         <v>27.456009839478661</v>
       </c>
-      <c r="Q10" s="69" t="s">
+      <c r="Q10" s="42" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       <c r="A11" s="14">
         <v>1.45</v>
       </c>
-      <c r="B11" s="65">
+      <c r="B11" s="38">
         <v>16</v>
       </c>
       <c r="C11" s="14">
@@ -1742,7 +1742,7 @@
         <f t="shared" si="1"/>
         <v>23.2</v>
       </c>
-      <c r="F11" s="61">
+      <c r="F11" s="34">
         <v>8.3333333333333339</v>
       </c>
       <c r="G11" s="16">
@@ -1777,14 +1777,14 @@
         <f>0.32*(K11*45/55+15)</f>
         <v>7.8294976906976901</v>
       </c>
-      <c r="O11" s="59">
+      <c r="O11" s="73">
         <v>5</v>
       </c>
       <c r="P11" s="13">
         <f t="shared" ref="P11:P16" si="10">L11</f>
         <v>27.026532191467624</v>
       </c>
-      <c r="Q11" s="69" t="s">
+      <c r="Q11" s="42" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       <c r="A12" s="25">
         <v>2.4500000000000002</v>
       </c>
-      <c r="B12" s="66">
+      <c r="B12" s="39">
         <v>17</v>
       </c>
       <c r="C12" s="26">
@@ -1807,7 +1807,7 @@
         <f t="shared" si="1"/>
         <v>40.200000000000003</v>
       </c>
-      <c r="F12" s="62">
+      <c r="F12" s="35">
         <v>15</v>
       </c>
       <c r="G12" s="27">
@@ -1842,12 +1842,12 @@
         <f t="shared" ref="N12:N16" si="12">0.32*(K12*45/55+15)</f>
         <v>9.5804875712332134</v>
       </c>
-      <c r="O12" s="59"/>
+      <c r="O12" s="73"/>
       <c r="P12" s="13">
         <f t="shared" si="10"/>
         <v>30.107451264062718</v>
       </c>
-      <c r="Q12" s="70" t="s">
+      <c r="Q12" s="56" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       <c r="A13" s="21">
         <v>3.45</v>
       </c>
-      <c r="B13" s="67">
+      <c r="B13" s="40">
         <v>17</v>
       </c>
       <c r="C13" s="21">
@@ -1870,7 +1870,7 @@
         <f t="shared" si="1"/>
         <v>57.2</v>
       </c>
-      <c r="F13" s="63">
+      <c r="F13" s="36">
         <v>19.3333333333333</v>
       </c>
       <c r="G13" s="22">
@@ -1905,18 +1905,18 @@
         <f t="shared" si="12"/>
         <v>10.405319020503489</v>
       </c>
-      <c r="O13" s="59"/>
+      <c r="O13" s="73"/>
       <c r="P13" s="13">
         <f t="shared" si="10"/>
         <v>31.358944263078541</v>
       </c>
-      <c r="Q13" s="71"/>
+      <c r="Q13" s="57"/>
     </row>
     <row r="14" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>4.45</v>
       </c>
-      <c r="B14" s="68">
+      <c r="B14" s="41">
         <v>17</v>
       </c>
       <c r="C14" s="1">
@@ -1931,7 +1931,7 @@
         <f t="shared" si="1"/>
         <v>74.2</v>
       </c>
-      <c r="F14" s="64">
+      <c r="F14" s="37">
         <v>22.666666666666668</v>
       </c>
       <c r="G14" s="2">
@@ -1966,12 +1966,12 @@
         <f t="shared" si="12"/>
         <v>10.890641940719346</v>
       </c>
-      <c r="O14" s="59"/>
+      <c r="O14" s="73"/>
       <c r="P14" s="13">
         <f t="shared" si="10"/>
         <v>32.052444298245355</v>
       </c>
-      <c r="Q14" s="71"/>
+      <c r="Q14" s="57"/>
       <c r="S14">
         <v>0.217</v>
       </c>
@@ -1980,7 +1980,7 @@
       <c r="A15" s="1">
         <v>5.45</v>
       </c>
-      <c r="B15" s="68">
+      <c r="B15" s="41">
         <v>17</v>
       </c>
       <c r="C15" s="1">
@@ -1995,7 +1995,7 @@
         <f t="shared" si="1"/>
         <v>91.2</v>
       </c>
-      <c r="F15" s="64">
+      <c r="F15" s="37">
         <v>26</v>
       </c>
       <c r="G15" s="2">
@@ -2030,18 +2030,18 @@
         <f t="shared" si="12"/>
         <v>11.348815895393484</v>
       </c>
-      <c r="O15" s="59"/>
+      <c r="O15" s="73"/>
       <c r="P15" s="13">
         <f t="shared" si="10"/>
         <v>32.682208038502324</v>
       </c>
-      <c r="Q15" s="71"/>
+      <c r="Q15" s="57"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>6.45</v>
       </c>
-      <c r="B16" s="68">
+      <c r="B16" s="41">
         <v>17</v>
       </c>
       <c r="C16" s="1">
@@ -2056,7 +2056,7 @@
         <f t="shared" si="1"/>
         <v>108.2</v>
       </c>
-      <c r="F16" s="64">
+      <c r="F16" s="37">
         <v>29.333333333333332</v>
       </c>
       <c r="G16" s="2">
@@ -2091,22 +2091,22 @@
         <f t="shared" si="12"/>
         <v>11.779425558195454</v>
       </c>
-      <c r="O16" s="59"/>
+      <c r="O16" s="73"/>
       <c r="P16" s="13">
         <f t="shared" si="10"/>
         <v>33.254289966218622</v>
       </c>
-      <c r="Q16" s="72"/>
+      <c r="Q16" s="58"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="19"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="33" t="s">
+      <c r="A18" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="33"/>
-      <c r="N18" s="73"/>
+      <c r="B18" s="44"/>
+      <c r="N18" s="43"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="32"/>

</xml_diff>

<commit_message>
casi terminado la primera parte de plantillas
</commit_message>
<xml_diff>
--- a/backend/templates/excel/plantilla_1.xlsx
+++ b/backend/templates/excel/plantilla_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecnologicodeantioquia-my.sharepoint.com/personal/paola_garcia44_correo_tdea_edu_co/Documents/Escritorio/Automatización geotecnica/automatizacion_geotecnica/backend/templates/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{622C883C-C2C7-4B70-A3F0-C530FA572C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{580A2FF4-72AA-40C2-ADF3-121DE9D6F21A}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{622C883C-C2C7-4B70-A3F0-C530FA572C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4399C9BE-B27E-4680-B4B9-39A1A370EA04}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -912,12 +912,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="17" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -981,9 +975,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -998,6 +989,15 @@
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1433,177 +1433,177 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="60"/>
-      <c r="P2" s="60"/>
-      <c r="Q2" s="61"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
+      <c r="Q2" s="59"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="62"/>
-      <c r="M3" s="62"/>
-      <c r="N3" s="62"/>
-      <c r="O3" s="62"/>
-      <c r="P3" s="62"/>
-      <c r="Q3" s="62"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="60"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
     </row>
     <row r="4" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="63"/>
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="64"/>
-      <c r="L4" s="64"/>
-      <c r="M4" s="64"/>
-      <c r="N4" s="64"/>
-      <c r="O4" s="64"/>
-      <c r="P4" s="64"/>
-      <c r="Q4" s="65"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="62"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="62"/>
+      <c r="N4" s="62"/>
+      <c r="O4" s="62"/>
+      <c r="P4" s="62"/>
+      <c r="Q4" s="63"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="66" t="s">
+      <c r="A5" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="66"/>
-      <c r="C5" s="67" t="s">
+      <c r="B5" s="64"/>
+      <c r="C5" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
-      <c r="L5" s="67"/>
-      <c r="M5" s="67"/>
-      <c r="N5" s="67"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
-      <c r="Q5" s="67"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="65"/>
+      <c r="M5" s="65"/>
+      <c r="N5" s="65"/>
+      <c r="O5" s="65"/>
+      <c r="P5" s="65"/>
+      <c r="Q5" s="65"/>
     </row>
     <row r="6" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="66" t="s">
+      <c r="A6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="66"/>
-      <c r="C6" s="68" t="s">
+      <c r="B6" s="64"/>
+      <c r="C6" s="71" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
-      <c r="N6" s="68"/>
-      <c r="O6" s="68"/>
-      <c r="P6" s="68"/>
-      <c r="Q6" s="68"/>
+      <c r="D6" s="71"/>
+      <c r="E6" s="71"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="71"/>
+      <c r="K6" s="71"/>
+      <c r="L6" s="71"/>
+      <c r="M6" s="71"/>
+      <c r="N6" s="71"/>
+      <c r="O6" s="71"/>
+      <c r="P6" s="71"/>
+      <c r="Q6" s="71"/>
     </row>
     <row r="7" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="72" t="s">
+      <c r="A7" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="72"/>
-      <c r="C7" s="45">
+      <c r="B7" s="69"/>
+      <c r="C7" s="72">
         <v>46112</v>
       </c>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="47" t="s">
+      <c r="D7" s="73"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="47"/>
+      <c r="G7" s="45"/>
       <c r="H7" s="10">
         <v>63.5</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="48" t="s">
+      <c r="J7" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="48"/>
-      <c r="L7" s="49" t="s">
+      <c r="K7" s="46"/>
+      <c r="L7" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="50"/>
-      <c r="N7" s="69" t="s">
+      <c r="M7" s="48"/>
+      <c r="N7" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="70"/>
-      <c r="P7" s="70"/>
-      <c r="Q7" s="71"/>
+      <c r="O7" s="67"/>
+      <c r="P7" s="67"/>
+      <c r="Q7" s="68"/>
     </row>
     <row r="8" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="72" t="s">
+      <c r="A8" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="72"/>
-      <c r="C8" s="53" t="s">
+      <c r="B8" s="69"/>
+      <c r="C8" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="54"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="47" t="s">
+      <c r="D8" s="52"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="47"/>
+      <c r="G8" s="45"/>
       <c r="H8" s="10">
         <v>0.76</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="48"/>
-      <c r="K8" s="48"/>
-      <c r="L8" s="51"/>
-      <c r="M8" s="52"/>
-      <c r="N8" s="69" t="s">
+      <c r="J8" s="46"/>
+      <c r="K8" s="46"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="50"/>
+      <c r="N8" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="O8" s="70"/>
-      <c r="P8" s="70"/>
-      <c r="Q8" s="71"/>
+      <c r="O8" s="67"/>
+      <c r="P8" s="67"/>
+      <c r="Q8" s="68"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -1777,7 +1777,7 @@
         <f>0.32*(K11*45/55+15)</f>
         <v>7.8294976906976901</v>
       </c>
-      <c r="O11" s="73">
+      <c r="O11" s="70">
         <v>5</v>
       </c>
       <c r="P11" s="13">
@@ -1842,12 +1842,12 @@
         <f t="shared" ref="N12:N16" si="12">0.32*(K12*45/55+15)</f>
         <v>9.5804875712332134</v>
       </c>
-      <c r="O12" s="73"/>
+      <c r="O12" s="70"/>
       <c r="P12" s="13">
         <f t="shared" si="10"/>
         <v>30.107451264062718</v>
       </c>
-      <c r="Q12" s="56" t="s">
+      <c r="Q12" s="54" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1905,12 +1905,12 @@
         <f t="shared" si="12"/>
         <v>10.405319020503489</v>
       </c>
-      <c r="O13" s="73"/>
+      <c r="O13" s="70"/>
       <c r="P13" s="13">
         <f t="shared" si="10"/>
         <v>31.358944263078541</v>
       </c>
-      <c r="Q13" s="57"/>
+      <c r="Q13" s="55"/>
     </row>
     <row r="14" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1966,12 +1966,12 @@
         <f t="shared" si="12"/>
         <v>10.890641940719346</v>
       </c>
-      <c r="O14" s="73"/>
+      <c r="O14" s="70"/>
       <c r="P14" s="13">
         <f t="shared" si="10"/>
         <v>32.052444298245355</v>
       </c>
-      <c r="Q14" s="57"/>
+      <c r="Q14" s="55"/>
       <c r="S14">
         <v>0.217</v>
       </c>
@@ -2030,12 +2030,12 @@
         <f t="shared" si="12"/>
         <v>11.348815895393484</v>
       </c>
-      <c r="O15" s="73"/>
+      <c r="O15" s="70"/>
       <c r="P15" s="13">
         <f t="shared" si="10"/>
         <v>32.682208038502324</v>
       </c>
-      <c r="Q15" s="57"/>
+      <c r="Q15" s="55"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -2091,12 +2091,12 @@
         <f t="shared" si="12"/>
         <v>11.779425558195454</v>
       </c>
-      <c r="O16" s="73"/>
+      <c r="O16" s="70"/>
       <c r="P16" s="13">
         <f t="shared" si="10"/>
         <v>33.254289966218622</v>
       </c>
-      <c r="Q16" s="58"/>
+      <c r="Q16" s="56"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="19"/>

</xml_diff>

<commit_message>
anexo varios documento en .zip
</commit_message>
<xml_diff>
--- a/backend/templates/excel/plantilla_1.xlsx
+++ b/backend/templates/excel/plantilla_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecnologicodeantioquia-my.sharepoint.com/personal/paola_garcia44_correo_tdea_edu_co/Documents/Escritorio/Automatización geotecnica/automatizacion_geotecnica/backend/templates/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{622C883C-C2C7-4B70-A3F0-C530FA572C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4399C9BE-B27E-4680-B4B9-39A1A370EA04}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{622C883C-C2C7-4B70-A3F0-C530FA572C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FBC09C9-A56D-48FE-97FC-44750A7D22E7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -878,33 +878,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -998,6 +971,33 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1433,177 +1433,177 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="58"/>
-      <c r="Q2" s="59"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="50"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="60"/>
-      <c r="M3" s="60"/>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="51"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="51"/>
+      <c r="N3" s="51"/>
+      <c r="O3" s="51"/>
+      <c r="P3" s="51"/>
+      <c r="Q3" s="51"/>
     </row>
     <row r="4" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="61"/>
-      <c r="B4" s="62"/>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="62"/>
-      <c r="L4" s="62"/>
-      <c r="M4" s="62"/>
-      <c r="N4" s="62"/>
-      <c r="O4" s="62"/>
-      <c r="P4" s="62"/>
-      <c r="Q4" s="63"/>
+      <c r="A4" s="52"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="53"/>
+      <c r="P4" s="53"/>
+      <c r="Q4" s="54"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="65" t="s">
+      <c r="B5" s="55"/>
+      <c r="C5" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="65"/>
-      <c r="J5" s="65"/>
-      <c r="K5" s="65"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="65"/>
-      <c r="N5" s="65"/>
-      <c r="O5" s="65"/>
-      <c r="P5" s="65"/>
-      <c r="Q5" s="65"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="56"/>
+      <c r="M5" s="56"/>
+      <c r="N5" s="56"/>
+      <c r="O5" s="56"/>
+      <c r="P5" s="56"/>
+      <c r="Q5" s="56"/>
     </row>
     <row r="6" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="64"/>
-      <c r="C6" s="71" t="s">
+      <c r="B6" s="55"/>
+      <c r="C6" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="71"/>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="71"/>
-      <c r="J6" s="71"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="71"/>
-      <c r="M6" s="71"/>
-      <c r="N6" s="71"/>
-      <c r="O6" s="71"/>
-      <c r="P6" s="71"/>
-      <c r="Q6" s="71"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
+      <c r="K6" s="62"/>
+      <c r="L6" s="62"/>
+      <c r="M6" s="62"/>
+      <c r="N6" s="62"/>
+      <c r="O6" s="62"/>
+      <c r="P6" s="62"/>
+      <c r="Q6" s="62"/>
     </row>
     <row r="7" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="69"/>
-      <c r="C7" s="72">
+      <c r="B7" s="60"/>
+      <c r="C7" s="63">
         <v>46112</v>
       </c>
-      <c r="D7" s="73"/>
-      <c r="E7" s="73"/>
-      <c r="F7" s="45" t="s">
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="45"/>
+      <c r="G7" s="36"/>
       <c r="H7" s="10">
         <v>63.5</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="46" t="s">
+      <c r="J7" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="46"/>
-      <c r="L7" s="47" t="s">
+      <c r="K7" s="37"/>
+      <c r="L7" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="48"/>
-      <c r="N7" s="66" t="s">
+      <c r="M7" s="39"/>
+      <c r="N7" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="67"/>
-      <c r="P7" s="67"/>
-      <c r="Q7" s="68"/>
+      <c r="O7" s="58"/>
+      <c r="P7" s="58"/>
+      <c r="Q7" s="59"/>
     </row>
     <row r="8" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="69"/>
-      <c r="C8" s="51" t="s">
+      <c r="B8" s="60"/>
+      <c r="C8" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="52"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="45" t="s">
+      <c r="D8" s="43"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="45"/>
+      <c r="G8" s="36"/>
       <c r="H8" s="10">
         <v>0.76</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="46"/>
-      <c r="K8" s="46"/>
-      <c r="L8" s="49"/>
-      <c r="M8" s="50"/>
-      <c r="N8" s="66" t="s">
+      <c r="J8" s="37"/>
+      <c r="K8" s="37"/>
+      <c r="L8" s="40"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="O8" s="67"/>
-      <c r="P8" s="67"/>
-      <c r="Q8" s="68"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="58"/>
+      <c r="Q8" s="59"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -1662,7 +1662,7 @@
       <c r="A10" s="14">
         <v>0.45</v>
       </c>
-      <c r="B10" s="38">
+      <c r="B10" s="65">
         <v>15</v>
       </c>
       <c r="C10" s="14">
@@ -1677,7 +1677,7 @@
         <f t="shared" ref="E10:E16" si="1">C10-D10</f>
         <v>6.75</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="69">
         <v>7</v>
       </c>
       <c r="G10" s="16">
@@ -1719,7 +1719,7 @@
         <f>L10</f>
         <v>27.456009839478661</v>
       </c>
-      <c r="Q10" s="42" t="s">
+      <c r="Q10" s="33" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       <c r="A11" s="14">
         <v>1.45</v>
       </c>
-      <c r="B11" s="38">
+      <c r="B11" s="65">
         <v>16</v>
       </c>
       <c r="C11" s="14">
@@ -1742,7 +1742,7 @@
         <f t="shared" si="1"/>
         <v>23.2</v>
       </c>
-      <c r="F11" s="34">
+      <c r="F11" s="70">
         <v>8.3333333333333339</v>
       </c>
       <c r="G11" s="16">
@@ -1777,14 +1777,14 @@
         <f>0.32*(K11*45/55+15)</f>
         <v>7.8294976906976901</v>
       </c>
-      <c r="O11" s="70">
+      <c r="O11" s="61">
         <v>5</v>
       </c>
       <c r="P11" s="13">
         <f t="shared" ref="P11:P16" si="10">L11</f>
         <v>27.026532191467624</v>
       </c>
-      <c r="Q11" s="42" t="s">
+      <c r="Q11" s="33" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       <c r="A12" s="25">
         <v>2.4500000000000002</v>
       </c>
-      <c r="B12" s="39">
+      <c r="B12" s="66">
         <v>17</v>
       </c>
       <c r="C12" s="26">
@@ -1807,7 +1807,7 @@
         <f t="shared" si="1"/>
         <v>40.200000000000003</v>
       </c>
-      <c r="F12" s="35">
+      <c r="F12" s="71">
         <v>15</v>
       </c>
       <c r="G12" s="27">
@@ -1842,12 +1842,12 @@
         <f t="shared" ref="N12:N16" si="12">0.32*(K12*45/55+15)</f>
         <v>9.5804875712332134</v>
       </c>
-      <c r="O12" s="70"/>
+      <c r="O12" s="61"/>
       <c r="P12" s="13">
         <f t="shared" si="10"/>
         <v>30.107451264062718</v>
       </c>
-      <c r="Q12" s="54" t="s">
+      <c r="Q12" s="45" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       <c r="A13" s="21">
         <v>3.45</v>
       </c>
-      <c r="B13" s="40">
+      <c r="B13" s="67">
         <v>17</v>
       </c>
       <c r="C13" s="21">
@@ -1870,7 +1870,7 @@
         <f t="shared" si="1"/>
         <v>57.2</v>
       </c>
-      <c r="F13" s="36">
+      <c r="F13" s="72">
         <v>19.3333333333333</v>
       </c>
       <c r="G13" s="22">
@@ -1905,18 +1905,18 @@
         <f t="shared" si="12"/>
         <v>10.405319020503489</v>
       </c>
-      <c r="O13" s="70"/>
+      <c r="O13" s="61"/>
       <c r="P13" s="13">
         <f t="shared" si="10"/>
         <v>31.358944263078541</v>
       </c>
-      <c r="Q13" s="55"/>
+      <c r="Q13" s="46"/>
     </row>
     <row r="14" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>4.45</v>
       </c>
-      <c r="B14" s="41">
+      <c r="B14" s="68">
         <v>17</v>
       </c>
       <c r="C14" s="1">
@@ -1931,7 +1931,7 @@
         <f t="shared" si="1"/>
         <v>74.2</v>
       </c>
-      <c r="F14" s="37">
+      <c r="F14" s="73">
         <v>22.666666666666668</v>
       </c>
       <c r="G14" s="2">
@@ -1966,12 +1966,12 @@
         <f t="shared" si="12"/>
         <v>10.890641940719346</v>
       </c>
-      <c r="O14" s="70"/>
+      <c r="O14" s="61"/>
       <c r="P14" s="13">
         <f t="shared" si="10"/>
         <v>32.052444298245355</v>
       </c>
-      <c r="Q14" s="55"/>
+      <c r="Q14" s="46"/>
       <c r="S14">
         <v>0.217</v>
       </c>
@@ -1980,7 +1980,7 @@
       <c r="A15" s="1">
         <v>5.45</v>
       </c>
-      <c r="B15" s="41">
+      <c r="B15" s="68">
         <v>17</v>
       </c>
       <c r="C15" s="1">
@@ -1995,7 +1995,7 @@
         <f t="shared" si="1"/>
         <v>91.2</v>
       </c>
-      <c r="F15" s="37">
+      <c r="F15" s="73">
         <v>26</v>
       </c>
       <c r="G15" s="2">
@@ -2030,18 +2030,18 @@
         <f t="shared" si="12"/>
         <v>11.348815895393484</v>
       </c>
-      <c r="O15" s="70"/>
+      <c r="O15" s="61"/>
       <c r="P15" s="13">
         <f t="shared" si="10"/>
         <v>32.682208038502324</v>
       </c>
-      <c r="Q15" s="55"/>
+      <c r="Q15" s="46"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>6.45</v>
       </c>
-      <c r="B16" s="41">
+      <c r="B16" s="68">
         <v>17</v>
       </c>
       <c r="C16" s="1">
@@ -2056,7 +2056,7 @@
         <f t="shared" si="1"/>
         <v>108.2</v>
       </c>
-      <c r="F16" s="37">
+      <c r="F16" s="73">
         <v>29.333333333333332</v>
       </c>
       <c r="G16" s="2">
@@ -2091,22 +2091,22 @@
         <f t="shared" si="12"/>
         <v>11.779425558195454</v>
       </c>
-      <c r="O16" s="70"/>
+      <c r="O16" s="61"/>
       <c r="P16" s="13">
         <f t="shared" si="10"/>
         <v>33.254289966218622</v>
       </c>
-      <c r="Q16" s="56"/>
+      <c r="Q16" s="47"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="19"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="44" t="s">
+      <c r="A18" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="44"/>
-      <c r="N18" s="43"/>
+      <c r="B18" s="35"/>
+      <c r="N18" s="34"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="32"/>

</xml_diff>

<commit_message>
tercera plantila casi lista falta cambiar unos datos
</commit_message>
<xml_diff>
--- a/backend/templates/excel/plantilla_1.xlsx
+++ b/backend/templates/excel/plantilla_1.xlsx
@@ -882,10 +882,97 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -910,93 +997,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1433,140 +1433,140 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="49"/>
-      <c r="Q2" s="50"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="48"/>
+      <c r="N2" s="48"/>
+      <c r="O2" s="48"/>
+      <c r="P2" s="48"/>
+      <c r="Q2" s="49"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
-      <c r="L3" s="51"/>
-      <c r="M3" s="51"/>
-      <c r="N3" s="51"/>
-      <c r="O3" s="51"/>
-      <c r="P3" s="51"/>
-      <c r="Q3" s="51"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="50"/>
+      <c r="L3" s="50"/>
+      <c r="M3" s="50"/>
+      <c r="N3" s="50"/>
+      <c r="O3" s="50"/>
+      <c r="P3" s="50"/>
+      <c r="Q3" s="50"/>
     </row>
     <row r="4" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="52"/>
-      <c r="B4" s="53"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
-      <c r="K4" s="53"/>
-      <c r="L4" s="53"/>
-      <c r="M4" s="53"/>
-      <c r="N4" s="53"/>
-      <c r="O4" s="53"/>
-      <c r="P4" s="53"/>
-      <c r="Q4" s="54"/>
+      <c r="A4" s="51"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="52"/>
+      <c r="I4" s="52"/>
+      <c r="J4" s="52"/>
+      <c r="K4" s="52"/>
+      <c r="L4" s="52"/>
+      <c r="M4" s="52"/>
+      <c r="N4" s="52"/>
+      <c r="O4" s="52"/>
+      <c r="P4" s="52"/>
+      <c r="Q4" s="53"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="55" t="s">
+      <c r="A5" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="55"/>
-      <c r="C5" s="56" t="s">
+      <c r="B5" s="54"/>
+      <c r="C5" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
-      <c r="K5" s="56"/>
-      <c r="L5" s="56"/>
-      <c r="M5" s="56"/>
-      <c r="N5" s="56"/>
-      <c r="O5" s="56"/>
-      <c r="P5" s="56"/>
-      <c r="Q5" s="56"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="55"/>
+      <c r="I5" s="55"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="55"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="55"/>
+      <c r="O5" s="55"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="55"/>
     </row>
     <row r="6" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="55"/>
-      <c r="C6" s="62" t="s">
+      <c r="B6" s="54"/>
+      <c r="C6" s="56" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="62"/>
-      <c r="H6" s="62"/>
-      <c r="I6" s="62"/>
-      <c r="J6" s="62"/>
-      <c r="K6" s="62"/>
-      <c r="L6" s="62"/>
-      <c r="M6" s="62"/>
-      <c r="N6" s="62"/>
-      <c r="O6" s="62"/>
-      <c r="P6" s="62"/>
-      <c r="Q6" s="62"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="56"/>
+      <c r="M6" s="56"/>
+      <c r="N6" s="56"/>
+      <c r="O6" s="56"/>
+      <c r="P6" s="56"/>
+      <c r="Q6" s="56"/>
     </row>
     <row r="7" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="60" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="60"/>
-      <c r="C7" s="63">
+      <c r="C7" s="64">
         <v>46112</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="64"/>
-      <c r="F7" s="36" t="s">
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="36"/>
+      <c r="G7" s="61"/>
       <c r="H7" s="10">
         <v>63.5</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="37" t="s">
+      <c r="J7" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="37"/>
-      <c r="L7" s="38" t="s">
+      <c r="K7" s="66"/>
+      <c r="L7" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="39"/>
+      <c r="M7" s="68"/>
       <c r="N7" s="57" t="s">
         <v>18</v>
       </c>
@@ -1579,25 +1579,25 @@
         <v>14</v>
       </c>
       <c r="B8" s="60"/>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="71" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="43"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="36" t="s">
+      <c r="D8" s="72"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="36"/>
+      <c r="G8" s="61"/>
       <c r="H8" s="10">
         <v>0.76</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="37"/>
-      <c r="K8" s="37"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="41"/>
+      <c r="J8" s="66"/>
+      <c r="K8" s="66"/>
+      <c r="L8" s="69"/>
+      <c r="M8" s="70"/>
       <c r="N8" s="57" t="s">
         <v>20</v>
       </c>
@@ -1662,7 +1662,7 @@
       <c r="A10" s="14">
         <v>0.45</v>
       </c>
-      <c r="B10" s="65">
+      <c r="B10" s="35">
         <v>15</v>
       </c>
       <c r="C10" s="14">
@@ -1677,7 +1677,7 @@
         <f t="shared" ref="E10:E16" si="1">C10-D10</f>
         <v>6.75</v>
       </c>
-      <c r="F10" s="69">
+      <c r="F10" s="39">
         <v>7</v>
       </c>
       <c r="G10" s="16">
@@ -1727,7 +1727,7 @@
       <c r="A11" s="14">
         <v>1.45</v>
       </c>
-      <c r="B11" s="65">
+      <c r="B11" s="35">
         <v>16</v>
       </c>
       <c r="C11" s="14">
@@ -1742,7 +1742,7 @@
         <f t="shared" si="1"/>
         <v>23.2</v>
       </c>
-      <c r="F11" s="70">
+      <c r="F11" s="40">
         <v>8.3333333333333339</v>
       </c>
       <c r="G11" s="16">
@@ -1777,7 +1777,7 @@
         <f>0.32*(K11*45/55+15)</f>
         <v>7.8294976906976901</v>
       </c>
-      <c r="O11" s="61">
+      <c r="O11" s="62">
         <v>5</v>
       </c>
       <c r="P11" s="13">
@@ -1792,7 +1792,7 @@
       <c r="A12" s="25">
         <v>2.4500000000000002</v>
       </c>
-      <c r="B12" s="66">
+      <c r="B12" s="36">
         <v>17</v>
       </c>
       <c r="C12" s="26">
@@ -1807,7 +1807,7 @@
         <f t="shared" si="1"/>
         <v>40.200000000000003</v>
       </c>
-      <c r="F12" s="71">
+      <c r="F12" s="41">
         <v>15</v>
       </c>
       <c r="G12" s="27">
@@ -1842,12 +1842,12 @@
         <f t="shared" ref="N12:N16" si="12">0.32*(K12*45/55+15)</f>
         <v>9.5804875712332134</v>
       </c>
-      <c r="O12" s="61"/>
+      <c r="O12" s="62"/>
       <c r="P12" s="13">
         <f t="shared" si="10"/>
         <v>30.107451264062718</v>
       </c>
-      <c r="Q12" s="45" t="s">
+      <c r="Q12" s="44" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       <c r="A13" s="21">
         <v>3.45</v>
       </c>
-      <c r="B13" s="67">
+      <c r="B13" s="37">
         <v>17</v>
       </c>
       <c r="C13" s="21">
@@ -1870,7 +1870,7 @@
         <f t="shared" si="1"/>
         <v>57.2</v>
       </c>
-      <c r="F13" s="72">
+      <c r="F13" s="42">
         <v>19.3333333333333</v>
       </c>
       <c r="G13" s="22">
@@ -1905,18 +1905,18 @@
         <f t="shared" si="12"/>
         <v>10.405319020503489</v>
       </c>
-      <c r="O13" s="61"/>
+      <c r="O13" s="62"/>
       <c r="P13" s="13">
         <f t="shared" si="10"/>
         <v>31.358944263078541</v>
       </c>
-      <c r="Q13" s="46"/>
+      <c r="Q13" s="45"/>
     </row>
     <row r="14" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>4.45</v>
       </c>
-      <c r="B14" s="68">
+      <c r="B14" s="38">
         <v>17</v>
       </c>
       <c r="C14" s="1">
@@ -1931,7 +1931,7 @@
         <f t="shared" si="1"/>
         <v>74.2</v>
       </c>
-      <c r="F14" s="73">
+      <c r="F14" s="43">
         <v>22.666666666666668</v>
       </c>
       <c r="G14" s="2">
@@ -1966,12 +1966,12 @@
         <f t="shared" si="12"/>
         <v>10.890641940719346</v>
       </c>
-      <c r="O14" s="61"/>
+      <c r="O14" s="62"/>
       <c r="P14" s="13">
         <f t="shared" si="10"/>
         <v>32.052444298245355</v>
       </c>
-      <c r="Q14" s="46"/>
+      <c r="Q14" s="45"/>
       <c r="S14">
         <v>0.217</v>
       </c>
@@ -1980,7 +1980,7 @@
       <c r="A15" s="1">
         <v>5.45</v>
       </c>
-      <c r="B15" s="68">
+      <c r="B15" s="38">
         <v>17</v>
       </c>
       <c r="C15" s="1">
@@ -1995,7 +1995,7 @@
         <f t="shared" si="1"/>
         <v>91.2</v>
       </c>
-      <c r="F15" s="73">
+      <c r="F15" s="43">
         <v>26</v>
       </c>
       <c r="G15" s="2">
@@ -2030,18 +2030,18 @@
         <f t="shared" si="12"/>
         <v>11.348815895393484</v>
       </c>
-      <c r="O15" s="61"/>
+      <c r="O15" s="62"/>
       <c r="P15" s="13">
         <f t="shared" si="10"/>
         <v>32.682208038502324</v>
       </c>
-      <c r="Q15" s="46"/>
+      <c r="Q15" s="45"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>6.45</v>
       </c>
-      <c r="B16" s="68">
+      <c r="B16" s="38">
         <v>17</v>
       </c>
       <c r="C16" s="1">
@@ -2056,7 +2056,7 @@
         <f t="shared" si="1"/>
         <v>108.2</v>
       </c>
-      <c r="F16" s="73">
+      <c r="F16" s="43">
         <v>29.333333333333332</v>
       </c>
       <c r="G16" s="2">
@@ -2091,21 +2091,21 @@
         <f t="shared" si="12"/>
         <v>11.779425558195454</v>
       </c>
-      <c r="O16" s="61"/>
+      <c r="O16" s="62"/>
       <c r="P16" s="13">
         <f t="shared" si="10"/>
         <v>33.254289966218622</v>
       </c>
-      <c r="Q16" s="47"/>
+      <c r="Q16" s="46"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="19"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
+      <c r="A18" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="35"/>
+      <c r="B18" s="63"/>
       <c r="N18" s="34"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -2139,6 +2139,12 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="J7:K8"/>
+    <mergeCell ref="L7:M8"/>
+    <mergeCell ref="C8:E8"/>
     <mergeCell ref="Q12:Q16"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A3:Q3"/>
@@ -2153,12 +2159,6 @@
     <mergeCell ref="N8:Q8"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="O11:O16"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="J7:K8"/>
-    <mergeCell ref="L7:M8"/>
-    <mergeCell ref="C8:E8"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.55118110236220474" bottom="0.55118110236220474" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>